<commit_message>
Add PDF presentation upload and block31 mapping
</commit_message>
<xml_diff>
--- a/Данные для разработки.xlsx
+++ b/Данные для разработки.xlsx
@@ -1686,7 +1686,7 @@
         <v>5</v>
       </c>
       <c r="N2" s="3">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="O2" s="3">
         <v>7</v>
@@ -1751,7 +1751,7 @@
         <v>6</v>
       </c>
       <c r="N3" s="3">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="O3" s="3">
         <v>8</v>
@@ -1816,7 +1816,7 @@
         <v>7</v>
       </c>
       <c r="N4" s="3">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="O4" s="3">
         <v>6</v>
@@ -1881,7 +1881,7 @@
         <v>4</v>
       </c>
       <c r="N5" s="3">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="O5" s="3">
         <v>9</v>
@@ -1946,7 +1946,7 @@
         <v>5</v>
       </c>
       <c r="N6" s="3">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="O6" s="3">
         <v>8</v>
@@ -2011,7 +2011,7 @@
         <v>3</v>
       </c>
       <c r="N7" s="3">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="O7" s="3">
         <v>5</v>
@@ -2049,7 +2049,7 @@
         <v>5</v>
       </c>
       <c r="N8" s="3">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="O8" s="3">
         <v>7</v>
@@ -2087,7 +2087,7 @@
         <v>6</v>
       </c>
       <c r="N9" s="3">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="O9" s="3">
         <v>8</v>
@@ -2125,7 +2125,7 @@
         <v>7</v>
       </c>
       <c r="N10" s="3">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="O10" s="3">
         <v>6</v>
@@ -2163,7 +2163,7 @@
         <v>4</v>
       </c>
       <c r="N11" s="3">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="O11" s="3">
         <v>9</v>
@@ -2201,7 +2201,7 @@
         <v>5</v>
       </c>
       <c r="N12" s="3">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="O12" s="3">
         <v>8</v>
@@ -2239,7 +2239,7 @@
         <v>3</v>
       </c>
       <c r="N13" s="3">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="O13" s="3">
         <v>5</v>
@@ -2277,7 +2277,7 @@
         <v>5</v>
       </c>
       <c r="N14" s="3">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="O14" s="3">
         <v>7</v>
@@ -2315,7 +2315,7 @@
         <v>6</v>
       </c>
       <c r="N15" s="3">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="O15" s="3">
         <v>8</v>
@@ -2353,7 +2353,7 @@
         <v>7</v>
       </c>
       <c r="N16" s="3">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="O16" s="3">
         <v>6</v>
@@ -2391,7 +2391,7 @@
         <v>4</v>
       </c>
       <c r="N17" s="3">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="O17" s="3">
         <v>9</v>
@@ -2429,7 +2429,7 @@
         <v>5</v>
       </c>
       <c r="N18" s="3">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="O18" s="3">
         <v>8</v>
@@ -2467,7 +2467,7 @@
         <v>3</v>
       </c>
       <c r="N19" s="3">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="O19" s="3">
         <v>5</v>
@@ -2505,7 +2505,7 @@
         <v>5</v>
       </c>
       <c r="N20" s="3">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="O20" s="3">
         <v>7</v>
@@ -2543,7 +2543,7 @@
         <v>6</v>
       </c>
       <c r="N21" s="3">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="O21" s="3">
         <v>8</v>
@@ -2581,7 +2581,7 @@
         <v>7</v>
       </c>
       <c r="N22" s="3">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="O22" s="3">
         <v>6</v>
@@ -2619,7 +2619,7 @@
         <v>4</v>
       </c>
       <c r="N23" s="3">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="O23" s="3">
         <v>9</v>
@@ -2657,7 +2657,7 @@
         <v>5</v>
       </c>
       <c r="N24" s="3">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="O24" s="3">
         <v>8</v>
@@ -2695,7 +2695,7 @@
         <v>3</v>
       </c>
       <c r="N25" s="3">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="O25" s="3">
         <v>5</v>
@@ -2733,7 +2733,7 @@
         <v>5</v>
       </c>
       <c r="N26" s="3">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="O26" s="3">
         <v>7</v>
@@ -2771,7 +2771,7 @@
         <v>6</v>
       </c>
       <c r="N27" s="3">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="O27" s="3">
         <v>8</v>
@@ -2809,7 +2809,7 @@
         <v>7</v>
       </c>
       <c r="N28" s="3">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="O28" s="3">
         <v>6</v>
@@ -2847,7 +2847,7 @@
         <v>4</v>
       </c>
       <c r="N29" s="3">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="O29" s="3">
         <v>9</v>
@@ -2885,7 +2885,7 @@
         <v>5</v>
       </c>
       <c r="N30" s="3">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="O30" s="3">
         <v>8</v>
@@ -2923,7 +2923,7 @@
         <v>3</v>
       </c>
       <c r="N31" s="3">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="O31" s="3">
         <v>5</v>
@@ -2960,8 +2960,8 @@
       <c r="M32" s="27">
         <v>7</v>
       </c>
-      <c r="N32" s="25">
-        <v>28</v>
+      <c r="N32" s="3">
+        <v>52</v>
       </c>
       <c r="O32" s="3">
         <v>7</v>

</xml_diff>